<commit_message>
feat: Add Git LFS configuration for `index2.pdf` and capture push error logs.
</commit_message>
<xml_diff>
--- a/public/8-1 - BTS SIO - 2025 - Annexe 8-1 - Epreuve E5 - Tableau de synthèse (1).xlsx
+++ b/public/8-1 - BTS SIO - 2025 - Annexe 8-1 - Epreuve E5 - Tableau de synthèse (1).xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gabdo\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3294494235b341b4/Escritorio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01113F02-F186-4B98-B18D-9C8C6673A072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{01113F02-F186-4B98-B18D-9C8C6673A072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88CC4BBC-3666-453E-BF7C-B3D37C3AC850}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="43">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -137,25 +137,40 @@
     <t>TP Gestion de projet - Planification des activités, gestion des risques et réalisation de diagrammes de Gantt et PERT (Cas ESN Proj'Info et Schuman SARL).</t>
   </si>
   <si>
-    <t>TP Méthodes Agiles et SCRUM - Simulation de gestion de projet : rédaction de user stories, création d'un backlog produit et estimation des tâches avec le Planning Poker.</t>
-  </si>
-  <si>
     <t>TD Veille Informationnelle - Choix des thématiques, comparaison des outils et mise en place d'une démarche de veille automatisée assistée par l'IA (Feedly, Notion, IA).</t>
   </si>
   <si>
     <t>03/10/2025 al 12/12/2025</t>
   </si>
   <si>
-    <t>Développement de deux applications web (pour un centre médical et un casino) utilisant PHP, JavaScript et CSS.</t>
-  </si>
-  <si>
-    <t>19/05/25 au 04/06/25</t>
-  </si>
-  <si>
-    <t>Stage 2 (MP44) - Conception d'interfaces interactives (React.js) pour bornes intelligentes avec intégration d'IA (Google AI Studio), automatisation (Make) et déploiement continu (GitHub/Netlify).</t>
-  </si>
-  <si>
     <t>05/01/26 au 13/02/26</t>
+  </si>
+  <si>
+    <t>Développement de une application web (pour un centre médical) utilisant PHP, JavaScript et CSS.</t>
+  </si>
+  <si>
+    <t>Développement de une application web (pour un casino) utilisant PHP, JavaScript et CSS.</t>
+  </si>
+  <si>
+    <t>19/05/25 au 16/06/25</t>
+  </si>
+  <si>
+    <t>16/06/25 au 04/07/25</t>
+  </si>
+  <si>
+    <t>Creation d'une aplication pour les auto écoles (utilisant Reacht et TypeScrype)</t>
+  </si>
+  <si>
+    <t>conception des système d'automatisation de recuperation et tratement de donnes ( utilisant l'aplication Make)</t>
+  </si>
+  <si>
+    <t>15/12/2025 au 19/12/2025</t>
+  </si>
+  <si>
+    <t>Projet de un universe 3D pour de casque VR réalisé lors de la semaine de challenge</t>
+  </si>
+  <si>
+    <t>09/02/26 au 13/02/26</t>
   </si>
 </sst>
 </file>
@@ -697,6 +712,12 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -762,12 +783,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -785,6 +800,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1088,56 +1107,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="H1" s="22"/>
+      <c r="H1" s="24"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="29" t="s">
+      <c r="B3" s="26"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="24"/>
-      <c r="H3" s="30"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="32"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="26" t="s">
+      <c r="A4" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="28"/>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="29"/>
+      <c r="E4" s="30"/>
       <c r="F4" s="14" t="s">
         <v>8</v>
       </c>
@@ -1149,22 +1168,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="43" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
+      <c r="B5" s="44"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="45"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="39" t="s">
+      <c r="B6" s="41" t="s">
         <v>19</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1187,8 +1206,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="32"/>
-      <c r="B7" s="40"/>
+      <c r="A7" s="34"/>
+      <c r="B7" s="42"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
@@ -1244,16 +1263,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A8" s="33" t="s">
+      <c r="A8" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="34"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="35"/>
+      <c r="B8" s="36"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="36"/>
+      <c r="H8" s="37"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1299,7 +1318,7 @@
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="17"/>
-      <c r="E9" s="44" t="s">
+      <c r="E9" s="22" t="s">
         <v>29</v>
       </c>
       <c r="F9" s="17"/>
@@ -1349,7 +1368,7 @@
       <c r="C10" s="17"/>
       <c r="D10" s="17"/>
       <c r="E10" s="17"/>
-      <c r="F10" s="44" t="s">
+      <c r="F10" s="22" t="s">
         <v>29</v>
       </c>
       <c r="G10" s="17"/>
@@ -1392,17 +1411,25 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" s="10"/>
+        <v>41</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>40</v>
+      </c>
       <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="44" t="s">
+      <c r="D11" s="22" t="s">
         <v>29</v>
       </c>
+      <c r="E11" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="F11" s="22" t="s">
+        <v>29</v>
+      </c>
       <c r="G11" s="17"/>
-      <c r="H11" s="18"/>
+      <c r="H11" s="23" t="s">
+        <v>29</v>
+      </c>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1441,17 +1468,17 @@
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="49.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="10" t="s">
-        <v>33</v>
-      </c>
       <c r="C12" s="17"/>
-      <c r="D12" s="44"/>
+      <c r="D12" s="22"/>
       <c r="E12" s="17"/>
       <c r="F12" s="17"/>
       <c r="G12" s="17"/>
-      <c r="H12" s="45" t="s">
+      <c r="H12" s="23" t="s">
         <v>29</v>
       </c>
       <c r="I12"/>
@@ -1761,16 +1788,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A19" s="36" t="s">
+      <c r="A19" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="B19" s="37"/>
-      <c r="C19" s="37"/>
-      <c r="D19" s="37"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="37"/>
-      <c r="G19" s="37"/>
-      <c r="H19" s="38"/>
+      <c r="B19" s="39"/>
+      <c r="C19" s="39"/>
+      <c r="D19" s="39"/>
+      <c r="E19" s="39"/>
+      <c r="F19" s="39"/>
+      <c r="G19" s="39"/>
+      <c r="H19" s="40"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1812,15 +1839,15 @@
         <v>34</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C20" s="17"/>
       <c r="D20" s="17"/>
-      <c r="E20" s="44" t="s">
+      <c r="E20" s="22" t="s">
         <v>29</v>
       </c>
       <c r="F20" s="17"/>
-      <c r="G20" s="44" t="s">
+      <c r="G20" s="22" t="s">
         <v>29</v>
       </c>
       <c r="H20" s="18"/>
@@ -1861,13 +1888,23 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="11"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="17"/>
+      <c r="A21" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="C21" s="22" t="s">
+        <v>29</v>
+      </c>
       <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
+      <c r="E21" s="22" t="s">
+        <v>29</v>
+      </c>
       <c r="F21" s="17"/>
-      <c r="G21" s="17"/>
+      <c r="G21" s="22" t="s">
+        <v>29</v>
+      </c>
       <c r="H21" s="18"/>
       <c r="I21"/>
       <c r="J21"/>
@@ -2131,16 +2168,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A27" s="36" t="s">
+      <c r="A27" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="B27" s="37"/>
-      <c r="C27" s="37"/>
-      <c r="D27" s="37"/>
-      <c r="E27" s="37"/>
-      <c r="F27" s="37"/>
-      <c r="G27" s="37"/>
-      <c r="H27" s="38"/>
+      <c r="B27" s="39"/>
+      <c r="C27" s="39"/>
+      <c r="D27" s="39"/>
+      <c r="E27" s="39"/>
+      <c r="F27" s="39"/>
+      <c r="G27" s="39"/>
+      <c r="H27" s="40"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2179,20 +2216,20 @@
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="11" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="C28" s="44" t="s">
+        <v>33</v>
+      </c>
+      <c r="C28" s="22" t="s">
         <v>29</v>
       </c>
       <c r="D28" s="17"/>
-      <c r="E28" s="44" t="s">
+      <c r="E28" s="22" t="s">
         <v>29</v>
       </c>
       <c r="F28" s="17"/>
-      <c r="G28" s="44" t="s">
+      <c r="G28" s="22" t="s">
         <v>29</v>
       </c>
       <c r="H28" s="18"/>
@@ -2233,13 +2270,25 @@
       <c r="AQ28"/>
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="11"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="17"/>
+      <c r="A29" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C29" s="22" t="s">
+        <v>29</v>
+      </c>
       <c r="D29" s="17"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="17"/>
-      <c r="G29" s="17"/>
+      <c r="E29" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="F29" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="G29" s="22" t="s">
+        <v>29</v>
+      </c>
       <c r="H29" s="18"/>
       <c r="I29"/>
       <c r="J29"/>

</xml_diff>